<commit_message>
Criação do script SamsungTVPlus
</commit_message>
<xml_diff>
--- a/the_stream_remains_the_same/tabulacao_conteudo_final.xlsx
+++ b/the_stream_remains_the_same/tabulacao_conteudo_final.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B36"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -369,351 +369,241 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>10 Play</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="B2">
-        <v>13</v>
+        <v>104</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AnthymTV</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="B3">
-        <v>21</v>
+        <v>106</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Brasil - GitHub</t>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="B4">
-        <v>332</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Brasil - Pluto</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="B5">
-        <v>141</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Brasil - SamsungTVPlus</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="B6">
-        <v>78</v>
+        <v>116</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BumbleBeeTV</t>
+          <t>Denmark</t>
         </is>
       </c>
       <c r="B7">
-        <v>40</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Cineverse</t>
+          <t>Finland</t>
         </is>
       </c>
       <c r="B8">
-        <v>23</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Distro</t>
+          <t>France</t>
         </is>
       </c>
       <c r="B9">
-        <v>211</v>
+        <v>121</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>FreeMoviesPlus</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="B10">
-        <v>17</v>
+        <v>122</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>FreeTV</t>
+          <t>India</t>
         </is>
       </c>
       <c r="B11">
-        <v>85</v>
+        <v>122</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>GitHub</t>
+          <t>Ireland</t>
         </is>
       </c>
       <c r="B12">
-        <v>10542</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>HerogoTV</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="B13">
-        <v>101</v>
+        <v>127</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Igocast</t>
+          <t>Luxembourg</t>
         </is>
       </c>
       <c r="B14">
-        <v>25</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>KlowdTV</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="B15">
-        <v>81</v>
+        <v>31</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Legal - Brasil</t>
+          <t>Netherland</t>
         </is>
       </c>
       <c r="B16">
-        <v>4044</v>
+        <v>52</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>LG</t>
+          <t>New Zealand</t>
         </is>
       </c>
       <c r="B17">
-        <v>1251</v>
+        <v>81</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>LocalNow</t>
+          <t>Norway</t>
         </is>
       </c>
       <c r="B18">
-        <v>485</v>
+        <v>20</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="B19">
-        <v>564</v>
+        <v>18</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Plex</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="B20">
-        <v>621</v>
+        <v>104</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>PlutoTV</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="B21">
-        <v>2263</v>
+        <v>114</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>RakutenTV</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="B22">
-        <v>259</v>
+        <v>76</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>RakutenTV J.P</t>
+          <t>Switzerland</t>
         </is>
       </c>
       <c r="B23">
-        <v>39</v>
+        <v>137</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Redbox</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="B24">
-        <v>184</v>
+        <v>155</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>RewardedTV</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="B25">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>SamsungTVPlus</t>
-        </is>
-      </c>
-      <c r="B26">
-        <v>2016</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>SportsTV</t>
-        </is>
-      </c>
-      <c r="B27">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Tablo</t>
-        </is>
-      </c>
-      <c r="B28">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>The Roku</t>
-        </is>
-      </c>
-      <c r="B29">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>TubiTV</t>
-        </is>
-      </c>
-      <c r="B30">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Veely</t>
-        </is>
-      </c>
-      <c r="B31">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Vidaa</t>
-        </is>
-      </c>
-      <c r="B32">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>VizioTV</t>
-        </is>
-      </c>
-      <c r="B33">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Xiaomi</t>
-        </is>
-      </c>
-      <c r="B34">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Xumo</t>
-        </is>
-      </c>
-      <c r="B35">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Zeasn</t>
-        </is>
-      </c>
-      <c r="B36">
-        <v>40</v>
+        <v>330</v>
       </c>
     </row>
   </sheetData>

</xml_diff>